<commit_message>
update DQ report summary template and summary image for Spring 2026 Covid & RSV script updates.
</commit_message>
<xml_diff>
--- a/Scripts/Vacc HB DQ Summary template.xlsx
+++ b/Scripts/Vacc HB DQ Summary template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\stats\VaccineDM\Mike\Scripts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\stats\VaccineDM\Mike\vacc-dq-reporting\Scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54848327-2932-497E-A916-CE242811B5ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{962A1E68-6878-4334-9531-D19627D30493}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1488,6 +1488,107 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>30. All query data</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> - All records that appear in the above queries. (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>QueryType</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is listed in </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>column A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.) This can be used to focus on individual patients by filtering by </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>column D - patient_derived_upi_number</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, to see all data quality queries against them, rather than by query type.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>20. HZ Vacc given outwith age guidance</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> - Herpes zoster vaccination records where the patient is not of eligible age at 1st Sep of that year and are not in any other eligibility cohort.</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t>27. COV Vacc given outwith age guidance</t>
     </r>
     <r>
@@ -1498,108 +1599,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> - Covid-19 records, from 1st April 2025, where the patient is not age 75 or over at 30th Jun 2025 and are not in an eligibility cohort.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>30. All query data</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> - All records that appear in the above queries. (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>QueryType</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> is listed in </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>column A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">.) This can be used to focus on individual patients by filtering by </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>column D - patient_derived_upi_number</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, to see all data quality queries against them, rather than by query type.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>20. HZ Vacc given outwith age guidance</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> - Herpes zoster vaccination records where the patient is not of eligible age at 1st Sep of that year and are not in any other eligibility cohort.</t>
+      <t xml:space="preserve"> - Covid-19 records, from 1st April 2025, where the patient is not in an eligibility cohort.</t>
     </r>
   </si>
 </sst>
@@ -2368,7 +2368,7 @@
       <c r="B32" s="1"/>
       <c r="C32" s="6"/>
       <c r="D32" s="17" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E32" s="7"/>
       <c r="F32" s="1"/>
@@ -2427,11 +2427,11 @@
       <c r="E38" s="7"/>
       <c r="F38" s="1"/>
     </row>
-    <row r="39" spans="2:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B39" s="1"/>
       <c r="C39" s="6"/>
       <c r="D39" s="17" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E39" s="7"/>
       <c r="F39" s="1"/>
@@ -2458,7 +2458,7 @@
       <c r="B42" s="1"/>
       <c r="C42" s="6"/>
       <c r="D42" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E42" s="7"/>
       <c r="F42" s="1"/>

</xml_diff>